<commit_message>
update upload bank's name
</commit_message>
<xml_diff>
--- a/static/uploads/mau/capnhatstk/capnhatstk.xlsx
+++ b/static/uploads/mau/capnhatstk/capnhatstk.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Khanh\Desktop\HRM\static\uploads\mau\capnhatstk\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\HRM\static\uploads\mau\capnhatstk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C55F5DA-7959-477B-9508-80B0714F3CA3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46AEED85-2D90-47AB-A045-1D19F69FC74C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{6C1BFFFF-0B88-49C7-B58B-818760297612}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{6C1BFFFF-0B88-49C7-B58B-818760297612}"/>
   </bookViews>
   <sheets>
     <sheet name="taikhoan" sheetId="2" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="289" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="198">
   <si>
     <t>04818</t>
   </si>
@@ -607,13 +607,25 @@
   </si>
   <si>
     <t>NT2</t>
+  </si>
+  <si>
+    <t>Tên ngân hàng</t>
+  </si>
+  <si>
+    <t>Agribank</t>
+  </si>
+  <si>
+    <t>MB Bank</t>
+  </si>
+  <si>
+    <t>VietinBank</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -656,7 +668,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -677,6 +689,17 @@
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
@@ -700,7 +723,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1037,14 +1060,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5B451787-37C2-410D-B666-4681EA093AAF}">
-  <dimension ref="A1:C97"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <dimension ref="A1:D97"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5" style="6" customWidth="1"/>
-    <col min="2" max="3" width="21.625" style="5" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" style="5" customWidth="1"/>
+    <col min="2" max="3" width="21.6640625" style="5" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>192</v>
       </c>
@@ -1054,9 +1078,12 @@
       <c r="C1" s="4" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15">
-      <c r="A2" s="6" t="s">
+      <c r="D1" s="6" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1065,9 +1092,12 @@
       <c r="C2" s="2" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="15">
-      <c r="A3" s="6" t="s">
+      <c r="D2" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B3" s="1" t="s">
@@ -1076,9 +1106,12 @@
       <c r="C3" s="2" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="15">
-      <c r="A4" s="6" t="s">
+      <c r="D3" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B4" s="1" t="s">
@@ -1087,9 +1120,12 @@
       <c r="C4" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="15">
-      <c r="A5" s="6" t="s">
+      <c r="D4" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B5" s="1" t="s">
@@ -1098,9 +1134,12 @@
       <c r="C5" s="2" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="15">
-      <c r="A6" s="6" t="s">
+      <c r="D5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -1109,9 +1148,12 @@
       <c r="C6" s="2" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="15">
-      <c r="A7" s="6" t="s">
+      <c r="D6" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B7" s="1" t="s">
@@ -1120,9 +1162,12 @@
       <c r="C7" s="2" t="s">
         <v>101</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="15">
-      <c r="A8" s="6" t="s">
+      <c r="D7" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B8" s="1" t="s">
@@ -1131,9 +1176,12 @@
       <c r="C8" s="2" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="15">
-      <c r="A9" s="6" t="s">
+      <c r="D8" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B9" s="1" t="s">
@@ -1142,9 +1190,12 @@
       <c r="C9" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="15">
-      <c r="A10" s="6" t="s">
+      <c r="D9" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -1153,9 +1204,12 @@
       <c r="C10" s="2" t="s">
         <v>104</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="15">
-      <c r="A11" s="6" t="s">
+      <c r="D10" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B11" s="1" t="s">
@@ -1164,9 +1218,12 @@
       <c r="C11" s="2" t="s">
         <v>105</v>
       </c>
-    </row>
-    <row r="12" spans="1:3" ht="15">
-      <c r="A12" s="6" t="s">
+      <c r="D11" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B12" s="1" t="s">
@@ -1175,9 +1232,12 @@
       <c r="C12" s="2" t="s">
         <v>106</v>
       </c>
-    </row>
-    <row r="13" spans="1:3" ht="15">
-      <c r="A13" s="6" t="s">
+      <c r="D12" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A13" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B13" s="1" t="s">
@@ -1186,9 +1246,12 @@
       <c r="C13" s="2" t="s">
         <v>107</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" ht="15">
-      <c r="A14" s="6" t="s">
+      <c r="D13" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A14" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -1197,9 +1260,12 @@
       <c r="C14" s="2" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="15" spans="1:3" ht="15">
-      <c r="A15" s="6" t="s">
+      <c r="D14" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A15" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B15" s="1" t="s">
@@ -1208,9 +1274,12 @@
       <c r="C15" s="2" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="16" spans="1:3" ht="15">
-      <c r="A16" s="6" t="s">
+      <c r="D15" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A16" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B16" s="1" t="s">
@@ -1219,9 +1288,12 @@
       <c r="C16" s="2" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="17" spans="1:3" ht="15">
-      <c r="A17" s="6" t="s">
+      <c r="D16" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B17" s="1" t="s">
@@ -1230,9 +1302,12 @@
       <c r="C17" s="2" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="18" spans="1:3" ht="15">
-      <c r="A18" s="6" t="s">
+      <c r="D17" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B18" s="1" t="s">
@@ -1241,9 +1316,12 @@
       <c r="C18" s="2" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="19" spans="1:3" ht="15">
-      <c r="A19" s="6" t="s">
+      <c r="D18" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B19" s="1" t="s">
@@ -1252,9 +1330,12 @@
       <c r="C19" s="2" t="s">
         <v>113</v>
       </c>
-    </row>
-    <row r="20" spans="1:3" ht="15">
-      <c r="A20" s="6" t="s">
+      <c r="D19" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B20" s="1" t="s">
@@ -1263,9 +1344,12 @@
       <c r="C20" s="2" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="21" spans="1:3" ht="15">
-      <c r="A21" s="6" t="s">
+      <c r="D20" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B21" s="1" t="s">
@@ -1274,9 +1358,12 @@
       <c r="C21" s="2" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="22" spans="1:3" ht="15">
-      <c r="A22" s="6" t="s">
+      <c r="D21" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B22" s="1" t="s">
@@ -1285,9 +1372,12 @@
       <c r="C22" s="2" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="23" spans="1:3" ht="15">
-      <c r="A23" s="6" t="s">
+      <c r="D22" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B23" s="1" t="s">
@@ -1296,9 +1386,12 @@
       <c r="C23" s="2" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="24" spans="1:3" ht="15">
-      <c r="A24" s="6" t="s">
+      <c r="D23" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B24" s="1" t="s">
@@ -1307,9 +1400,12 @@
       <c r="C24" s="2" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" ht="15">
-      <c r="A25" s="6" t="s">
+      <c r="D24" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B25" s="1" t="s">
@@ -1318,9 +1414,12 @@
       <c r="C25" s="2" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="26" spans="1:3" ht="15">
-      <c r="A26" s="6" t="s">
+      <c r="D25" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B26" s="1" t="s">
@@ -1329,9 +1428,12 @@
       <c r="C26" s="2" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="27" spans="1:3" ht="15">
-      <c r="A27" s="6" t="s">
+      <c r="D26" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B27" s="1" t="s">
@@ -1340,9 +1442,12 @@
       <c r="C27" s="2" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="28" spans="1:3" ht="15">
-      <c r="A28" s="6" t="s">
+      <c r="D27" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B28" s="1" t="s">
@@ -1351,9 +1456,12 @@
       <c r="C28" s="2" t="s">
         <v>122</v>
       </c>
-    </row>
-    <row r="29" spans="1:3" ht="15">
-      <c r="A29" s="6" t="s">
+      <c r="D28" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B29" s="1" t="s">
@@ -1362,9 +1470,12 @@
       <c r="C29" s="2" t="s">
         <v>123</v>
       </c>
-    </row>
-    <row r="30" spans="1:3" ht="15">
-      <c r="A30" s="6" t="s">
+      <c r="D29" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A30" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B30" s="1" t="s">
@@ -1373,9 +1484,12 @@
       <c r="C30" s="2" t="s">
         <v>124</v>
       </c>
-    </row>
-    <row r="31" spans="1:3" ht="15">
-      <c r="A31" s="6" t="s">
+      <c r="D30" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B31" s="1" t="s">
@@ -1384,9 +1498,12 @@
       <c r="C31" s="2" t="s">
         <v>125</v>
       </c>
-    </row>
-    <row r="32" spans="1:3" ht="15">
-      <c r="A32" s="6" t="s">
+      <c r="D31" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B32" s="1" t="s">
@@ -1395,9 +1512,12 @@
       <c r="C32" s="2" t="s">
         <v>126</v>
       </c>
-    </row>
-    <row r="33" spans="1:3" ht="15">
-      <c r="A33" s="6" t="s">
+      <c r="D32" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A33" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B33" s="1" t="s">
@@ -1406,9 +1526,12 @@
       <c r="C33" s="2" t="s">
         <v>127</v>
       </c>
-    </row>
-    <row r="34" spans="1:3" ht="15">
-      <c r="A34" s="6" t="s">
+      <c r="D33" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A34" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B34" s="1" t="s">
@@ -1417,9 +1540,12 @@
       <c r="C34" s="2" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="35" spans="1:3" ht="15">
-      <c r="A35" s="6" t="s">
+      <c r="D34" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A35" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B35" s="1" t="s">
@@ -1428,9 +1554,12 @@
       <c r="C35" s="2" t="s">
         <v>129</v>
       </c>
-    </row>
-    <row r="36" spans="1:3" ht="15">
-      <c r="A36" s="6" t="s">
+      <c r="D35" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A36" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B36" s="1" t="s">
@@ -1439,9 +1568,12 @@
       <c r="C36" s="2" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="37" spans="1:3" ht="15">
-      <c r="A37" s="6" t="s">
+      <c r="D36" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A37" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B37" s="1" t="s">
@@ -1450,9 +1582,12 @@
       <c r="C37" s="2" t="s">
         <v>131</v>
       </c>
-    </row>
-    <row r="38" spans="1:3" ht="15">
-      <c r="A38" s="6" t="s">
+      <c r="D37" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A38" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B38" s="1" t="s">
@@ -1461,9 +1596,12 @@
       <c r="C38" s="2" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="39" spans="1:3" ht="15">
-      <c r="A39" s="6" t="s">
+      <c r="D38" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A39" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B39" s="1" t="s">
@@ -1472,9 +1610,12 @@
       <c r="C39" s="2" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="40" spans="1:3" ht="15">
-      <c r="A40" s="6" t="s">
+      <c r="D39" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B40" s="1" t="s">
@@ -1483,9 +1624,12 @@
       <c r="C40" s="3">
         <v>102882192239</v>
       </c>
-    </row>
-    <row r="41" spans="1:3" ht="15">
-      <c r="A41" s="6" t="s">
+      <c r="D40" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A41" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B41" s="1" t="s">
@@ -1494,9 +1638,12 @@
       <c r="C41" s="2" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="42" spans="1:3" ht="15">
-      <c r="A42" s="6" t="s">
+      <c r="D41" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A42" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B42" s="1" t="s">
@@ -1505,9 +1652,12 @@
       <c r="C42" s="2" t="s">
         <v>135</v>
       </c>
-    </row>
-    <row r="43" spans="1:3" ht="15">
-      <c r="A43" s="6" t="s">
+      <c r="D42" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A43" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B43" s="1" t="s">
@@ -1516,9 +1666,12 @@
       <c r="C43" s="2" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="44" spans="1:3" ht="15">
-      <c r="A44" s="6" t="s">
+      <c r="D43" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A44" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B44" s="1" t="s">
@@ -1527,9 +1680,12 @@
       <c r="C44" s="2" t="s">
         <v>137</v>
       </c>
-    </row>
-    <row r="45" spans="1:3" ht="15">
-      <c r="A45" s="6" t="s">
+      <c r="D44" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A45" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B45" s="1" t="s">
@@ -1538,9 +1694,12 @@
       <c r="C45" s="2" t="s">
         <v>138</v>
       </c>
-    </row>
-    <row r="46" spans="1:3" ht="15">
-      <c r="A46" s="6" t="s">
+      <c r="D45" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A46" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B46" s="1" t="s">
@@ -1549,9 +1708,12 @@
       <c r="C46" s="2" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="47" spans="1:3" ht="15">
-      <c r="A47" s="6" t="s">
+      <c r="D46" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A47" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B47" s="1" t="s">
@@ -1560,9 +1722,12 @@
       <c r="C47" s="2" t="s">
         <v>140</v>
       </c>
-    </row>
-    <row r="48" spans="1:3" ht="15">
-      <c r="A48" s="6" t="s">
+      <c r="D47" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A48" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B48" s="1" t="s">
@@ -1571,9 +1736,12 @@
       <c r="C48" s="2" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="49" spans="1:3" ht="15">
-      <c r="A49" s="6" t="s">
+      <c r="D48" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A49" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B49" s="1" t="s">
@@ -1582,9 +1750,12 @@
       <c r="C49" s="2" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="50" spans="1:3" ht="15">
-      <c r="A50" s="6" t="s">
+      <c r="D49" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A50" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B50" s="1" t="s">
@@ -1593,9 +1764,12 @@
       <c r="C50" s="2" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="51" spans="1:3" ht="15">
-      <c r="A51" s="6" t="s">
+      <c r="D50" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A51" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B51" s="1" t="s">
@@ -1604,9 +1778,12 @@
       <c r="C51" s="2" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="52" spans="1:3" ht="15">
-      <c r="A52" s="6" t="s">
+      <c r="D51" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A52" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B52" s="1" t="s">
@@ -1615,9 +1792,12 @@
       <c r="C52" s="2" t="s">
         <v>145</v>
       </c>
-    </row>
-    <row r="53" spans="1:3" ht="15">
-      <c r="A53" s="6" t="s">
+      <c r="D52" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A53" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B53" s="1" t="s">
@@ -1626,9 +1806,12 @@
       <c r="C53" s="2" t="s">
         <v>146</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" ht="15">
-      <c r="A54" s="6" t="s">
+      <c r="D53" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A54" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B54" s="1" t="s">
@@ -1637,9 +1820,12 @@
       <c r="C54" s="2" t="s">
         <v>147</v>
       </c>
-    </row>
-    <row r="55" spans="1:3" ht="15">
-      <c r="A55" s="6" t="s">
+      <c r="D54" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A55" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B55" s="1" t="s">
@@ -1648,9 +1834,12 @@
       <c r="C55" s="2" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="56" spans="1:3" ht="15">
-      <c r="A56" s="6" t="s">
+      <c r="D55" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A56" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B56" s="1" t="s">
@@ -1659,9 +1848,12 @@
       <c r="C56" s="2" t="s">
         <v>149</v>
       </c>
-    </row>
-    <row r="57" spans="1:3" ht="15">
-      <c r="A57" s="6" t="s">
+      <c r="D56" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A57" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B57" s="1" t="s">
@@ -1670,9 +1862,12 @@
       <c r="C57" s="2" t="s">
         <v>150</v>
       </c>
-    </row>
-    <row r="58" spans="1:3" ht="15">
-      <c r="A58" s="6" t="s">
+      <c r="D57" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A58" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B58" s="1" t="s">
@@ -1681,9 +1876,12 @@
       <c r="C58" s="2" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="59" spans="1:3" ht="15">
-      <c r="A59" s="6" t="s">
+      <c r="D58" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A59" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B59" s="1" t="s">
@@ -1692,9 +1890,12 @@
       <c r="C59" s="2" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="60" spans="1:3" ht="15">
-      <c r="A60" s="6" t="s">
+      <c r="D59" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A60" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B60" s="1" t="s">
@@ -1703,9 +1904,12 @@
       <c r="C60" s="2" t="s">
         <v>153</v>
       </c>
-    </row>
-    <row r="61" spans="1:3" ht="15">
-      <c r="A61" s="6" t="s">
+      <c r="D60" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B61" s="1" t="s">
@@ -1714,9 +1918,12 @@
       <c r="C61" s="2" t="s">
         <v>154</v>
       </c>
-    </row>
-    <row r="62" spans="1:3" ht="15">
-      <c r="A62" s="6" t="s">
+      <c r="D61" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A62" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B62" s="1" t="s">
@@ -1725,9 +1932,12 @@
       <c r="C62" s="2" t="s">
         <v>155</v>
       </c>
-    </row>
-    <row r="63" spans="1:3" ht="15">
-      <c r="A63" s="6" t="s">
+      <c r="D62" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A63" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B63" s="1" t="s">
@@ -1736,9 +1946,12 @@
       <c r="C63" s="2" t="s">
         <v>156</v>
       </c>
-    </row>
-    <row r="64" spans="1:3" ht="15">
-      <c r="A64" s="6" t="s">
+      <c r="D63" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A64" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B64" s="1" t="s">
@@ -1747,9 +1960,12 @@
       <c r="C64" s="2" t="s">
         <v>157</v>
       </c>
-    </row>
-    <row r="65" spans="1:3" ht="15">
-      <c r="A65" s="6" t="s">
+      <c r="D64" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A65" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B65" s="1" t="s">
@@ -1758,9 +1974,12 @@
       <c r="C65" s="2" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="66" spans="1:3" ht="15">
-      <c r="A66" s="6" t="s">
+      <c r="D65" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A66" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B66" s="1" t="s">
@@ -1769,9 +1988,12 @@
       <c r="C66" s="2" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="67" spans="1:3" ht="15">
-      <c r="A67" s="6" t="s">
+      <c r="D66" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A67" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B67" s="1" t="s">
@@ -1780,9 +2002,12 @@
       <c r="C67" s="2" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="68" spans="1:3" ht="15">
-      <c r="A68" s="6" t="s">
+      <c r="D67" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A68" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B68" s="1" t="s">
@@ -1791,9 +2016,12 @@
       <c r="C68" s="2" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="69" spans="1:3" ht="15">
-      <c r="A69" s="6" t="s">
+      <c r="D68" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A69" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B69" s="1" t="s">
@@ -1802,9 +2030,12 @@
       <c r="C69" s="2" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="70" spans="1:3" ht="15">
-      <c r="A70" s="6" t="s">
+      <c r="D69" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A70" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B70" s="1" t="s">
@@ -1813,9 +2044,12 @@
       <c r="C70" s="2" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="71" spans="1:3" ht="15">
-      <c r="A71" s="6" t="s">
+      <c r="D70" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A71" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B71" s="1" t="s">
@@ -1824,9 +2058,12 @@
       <c r="C71" s="3">
         <v>104882190172</v>
       </c>
-    </row>
-    <row r="72" spans="1:3" ht="15">
-      <c r="A72" s="6" t="s">
+      <c r="D71" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A72" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B72" s="1" t="s">
@@ -1835,9 +2072,12 @@
       <c r="C72" s="2" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="73" spans="1:3" ht="15">
-      <c r="A73" s="6" t="s">
+      <c r="D72" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A73" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B73" s="1" t="s">
@@ -1846,9 +2086,12 @@
       <c r="C73" s="2" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="74" spans="1:3" ht="15">
-      <c r="A74" s="6" t="s">
+      <c r="D73" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A74" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B74" s="1" t="s">
@@ -1857,9 +2100,12 @@
       <c r="C74" s="2" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="75" spans="1:3" ht="15">
-      <c r="A75" s="6" t="s">
+      <c r="D74" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A75" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B75" s="1" t="s">
@@ -1868,9 +2114,12 @@
       <c r="C75" s="2" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="76" spans="1:3" ht="15">
-      <c r="A76" s="6" t="s">
+      <c r="D75" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A76" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B76" s="1" t="s">
@@ -1879,9 +2128,12 @@
       <c r="C76" s="2" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="77" spans="1:3" ht="15">
-      <c r="A77" s="6" t="s">
+      <c r="D76" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A77" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B77" s="1" t="s">
@@ -1890,9 +2142,12 @@
       <c r="C77" s="2" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="78" spans="1:3" ht="15">
-      <c r="A78" s="6" t="s">
+      <c r="D77" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A78" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B78" s="1" t="s">
@@ -1901,9 +2156,12 @@
       <c r="C78" s="2" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="79" spans="1:3" ht="15">
-      <c r="A79" s="6" t="s">
+      <c r="D78" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A79" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B79" s="1" t="s">
@@ -1912,9 +2170,12 @@
       <c r="C79" s="2" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="80" spans="1:3" ht="15">
-      <c r="A80" s="6" t="s">
+      <c r="D79" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A80" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B80" s="1" t="s">
@@ -1923,9 +2184,12 @@
       <c r="C80" s="2" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="81" spans="1:3" ht="15">
-      <c r="A81" s="6" t="s">
+      <c r="D80" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A81" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B81" s="1" t="s">
@@ -1934,9 +2198,12 @@
       <c r="C81" s="2" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="82" spans="1:3" ht="15">
-      <c r="A82" s="6" t="s">
+      <c r="D81" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A82" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B82" s="1" t="s">
@@ -1945,9 +2212,12 @@
       <c r="C82" s="2" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="83" spans="1:3" ht="15">
-      <c r="A83" s="6" t="s">
+      <c r="D82" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A83" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B83" s="1" t="s">
@@ -1956,9 +2226,12 @@
       <c r="C83" s="2" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="84" spans="1:3" ht="15">
-      <c r="A84" s="6" t="s">
+      <c r="D83" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A84" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B84" s="1" t="s">
@@ -1967,9 +2240,12 @@
       <c r="C84" s="2" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="85" spans="1:3" ht="15">
-      <c r="A85" s="6" t="s">
+      <c r="D84" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A85" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B85" s="1" t="s">
@@ -1978,9 +2254,12 @@
       <c r="C85" s="2" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="86" spans="1:3" ht="15">
-      <c r="A86" s="6" t="s">
+      <c r="D85" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A86" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B86" s="1" t="s">
@@ -1989,9 +2268,12 @@
       <c r="C86" s="2" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="87" spans="1:3" ht="15">
-      <c r="A87" s="6" t="s">
+      <c r="D86" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A87" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B87" s="1" t="s">
@@ -2000,9 +2282,12 @@
       <c r="C87" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="88" spans="1:3" ht="15">
-      <c r="A88" s="6" t="s">
+      <c r="D87" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A88" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B88" s="1" t="s">
@@ -2011,9 +2296,12 @@
       <c r="C88" s="2" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="89" spans="1:3" ht="15">
-      <c r="A89" s="6" t="s">
+      <c r="D88" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A89" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B89" s="1" t="s">
@@ -2022,9 +2310,12 @@
       <c r="C89" s="2" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="90" spans="1:3" ht="15">
-      <c r="A90" s="6" t="s">
+      <c r="D89" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A90" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B90" s="1" t="s">
@@ -2033,9 +2324,12 @@
       <c r="C90" s="2" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="91" spans="1:3" ht="15">
-      <c r="A91" s="6" t="s">
+      <c r="D90" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A91" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B91" s="1" t="s">
@@ -2044,9 +2338,12 @@
       <c r="C91" s="2" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="92" spans="1:3" ht="15">
-      <c r="A92" s="6" t="s">
+      <c r="D91" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A92" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B92" s="1" t="s">
@@ -2055,9 +2352,12 @@
       <c r="C92" s="2" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="93" spans="1:3" ht="15">
-      <c r="A93" s="6" t="s">
+      <c r="D92" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A93" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B93" s="1" t="s">
@@ -2066,9 +2366,12 @@
       <c r="C93" s="2" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="94" spans="1:3" ht="15">
-      <c r="A94" s="6" t="s">
+      <c r="D93" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="94" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A94" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B94" s="1" t="s">
@@ -2077,9 +2380,12 @@
       <c r="C94" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="95" spans="1:3" ht="15">
-      <c r="A95" s="6" t="s">
+      <c r="D94" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="95" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A95" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B95" s="1" t="s">
@@ -2088,9 +2394,12 @@
       <c r="C95" s="2" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="96" spans="1:3" ht="15">
-      <c r="A96" s="6" t="s">
+      <c r="D95" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="96" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A96" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B96" s="1" t="s">
@@ -2099,9 +2408,12 @@
       <c r="C96" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="97" spans="1:3" ht="15">
-      <c r="A97" s="6" t="s">
+      <c r="D96" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="97" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A97" s="5" t="s">
         <v>193</v>
       </c>
       <c r="B97" s="1" t="s">
@@ -2109,6 +2421,9 @@
       </c>
       <c r="C97" s="2" t="s">
         <v>189</v>
+      </c>
+      <c r="D97" t="s">
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>